<commit_message>
feat: new data structure for schedules + services
</commit_message>
<xml_diff>
--- a/client/public/templates/servicos.xlsx
+++ b/client/public/templates/servicos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ScopeSystem\client\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{429E36AF-04B5-4D2B-BECF-C6AA15FCC0B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED229618-5B49-487A-A302-CBFF4F56B371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{295BCE0E-7CE5-488C-86BB-3A01F9C37A3F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
   <si>
     <t>Placa</t>
   </si>
@@ -135,13 +135,64 @@
   </si>
   <si>
     <t>BOT</t>
+  </si>
+  <si>
+    <t>NumeroPedido</t>
+  </si>
+  <si>
+    <t>DataPedido</t>
+  </si>
+  <si>
+    <t>DataAgendamento</t>
+  </si>
+  <si>
+    <t>Responsavel</t>
+  </si>
+  <si>
+    <t>Condutor</t>
+  </si>
+  <si>
+    <t>GrupoVeiculo</t>
+  </si>
+  <si>
+    <t>Situacao</t>
+  </si>
+  <si>
+    <t>LocalServico</t>
+  </si>
+  <si>
+    <t>Motivo</t>
+  </si>
+  <si>
+    <t>Observacoes Gerais</t>
+  </si>
+  <si>
+    <t>Gabriel Barbosa</t>
+  </si>
+  <si>
+    <t>jose</t>
+  </si>
+  <si>
+    <t>rac</t>
+  </si>
+  <si>
+    <t>aguardando tecnico</t>
+  </si>
+  <si>
+    <t>teste</t>
+  </si>
+  <si>
+    <t>recall</t>
+  </si>
+  <si>
+    <t>obs</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -163,8 +214,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -186,6 +244,11 @@
       <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -211,12 +274,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="2"/>
@@ -227,9 +291,14 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
     <cellStyle name="40% - Ênfase1" xfId="2" builtinId="31"/>
+    <cellStyle name="Neutro" xfId="3" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Ruim" xfId="1" builtinId="27"/>
   </cellStyles>
@@ -578,7 +647,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F6C1C4B-5DDD-4FDE-9412-4F170193696F}">
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:AD2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.08984375" customWidth="1"/>
@@ -594,10 +663,14 @@
     <col min="13" max="13" width="8.6328125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="20.1796875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="16.08984375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="20.1796875" customWidth="1"/>
+    <col min="21" max="22" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -655,8 +728,39 @@
       <c r="S1" s="2" t="s">
         <v>31</v>
       </c>
+      <c r="T1" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="U1" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="V1" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="W1" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="X1" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y1" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="Z1" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="AA1" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB1" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="AC1" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="AD1" s="6"/>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -707,6 +811,36 @@
       </c>
       <c r="Q2" t="s">
         <v>32</v>
+      </c>
+      <c r="T2">
+        <v>342</v>
+      </c>
+      <c r="U2" s="7">
+        <v>46144</v>
+      </c>
+      <c r="V2" s="7">
+        <v>46147</v>
+      </c>
+      <c r="W2" t="s">
+        <v>43</v>
+      </c>
+      <c r="X2" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>46</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>